<commit_message>
refactored review sheet generation code into generate_review.py
</commit_message>
<xml_diff>
--- a/Results/V2/information_elements_manual_review.xlsx
+++ b/Results/V2/information_elements_manual_review.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -585,36 +585,118 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
+        <v>135</v>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>Wikimedia Commons</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>V2</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>HC_HP</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>Open App, swipe left four times, tap YES, tap Skip, tap YES, open the navigation drawer, select Explore, tap a picture, swipe up twice, tap a category, and tap Parent Categories to reach the Category screen in the Parent Categories tab; clicking the Parent Categories tab results in a blank page, but the Parent Categories of the current category should be displayed.</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>Title: Category details "PARENT CATEGORIES" tab shows a blank page
+Observed Behavior: On the CategoryDetailsActivity screen for a category, if the user taps the "PARENT CATEGORIES" tab, the app shows a blank page (no content displayed).
+Expected Behavior: The app should display the parent categories of the current category after tapping the "PARENT CATEGORIES" tab.</t>
+        </is>
+      </c>
+      <c r="G4" s="1" t="inlineStr">
+        <is>
+          <t>Buggy Behavior: see a blank page
+Triggering GUI Interaction: clicks the Parent Categories tab
+Triggering Screen Reference: Category screen, Parent Categories tab
+Correct Behavior: The Parent Categories of the current category should be displayed</t>
+        </is>
+      </c>
+      <c r="H4" s="1" t="inlineStr">
+        <is>
+          <t>Buggy Behavior: the app shows a blank page (no content displayed).
+Triggering GUI Interactions: the user taps the "PARENT CATEGORIES" tab
+Triggering Screen Reference: On the CategoryDetailsActivity screen for a category
+Correct Behavior: The app should display the parent categories of the current category after tapping the "PARENT CATEGORIES" tab.</t>
+        </is>
+      </c>
+      <c r="I4" s="1" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+      <c r="J4" s="1" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+      <c r="K4" s="1" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+      <c r="L4" s="1" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr"/>
+      <c r="B5" s="2" t="inlineStr"/>
+      <c r="C5" s="2" t="inlineStr"/>
+      <c r="D5" s="2" t="inlineStr"/>
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr"/>
+      <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr"/>
+      <c r="K5" s="2" t="inlineStr"/>
+      <c r="L5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="1" t="inlineStr">
+      <c r="B6" s="1" t="inlineStr">
         <is>
           <t>Family Finance</t>
         </is>
       </c>
-      <c r="C4" s="1" t="inlineStr">
+      <c r="C6" s="1" t="inlineStr">
         <is>
           <t>V2</t>
         </is>
       </c>
-      <c r="D4" s="1" t="inlineStr">
+      <c r="D6" s="1" t="inlineStr">
         <is>
           <t>MC_MP</t>
         </is>
       </c>
-      <c r="E4" s="1" t="inlineStr">
+      <c r="E6" s="1" t="inlineStr">
         <is>
           <t>Changing the report appearance from 'view values' to 'use percent values' results in the application crashing.</t>
         </is>
       </c>
-      <c r="F4" s="1" t="inlineStr">
+      <c r="F6" s="1" t="inlineStr">
         <is>
           <t>Title: Crash when enabling “Use percent values” in Reports &gt; Incomes by Articles display options
 Observed Behavior: On the Reports screen (Incomes by Articles tab), if the user opens the “Display” dialog and taps the “Use percent values” checkbox, the app crashes and shows a crash dialog/message: “Unfortunately, Family Finance has stopped.”
 Expected Behavior: The view should switch from “view values” to “use percent values” without crashing.</t>
         </is>
       </c>
-      <c r="G4" s="1" t="inlineStr">
+      <c r="G6" s="1" t="inlineStr">
         <is>
           <t>Buggy Behavior: the application crashes
 Triggering GUI Interaction: changes the appearance of the report from 'view values' to use percent values'
@@ -622,7 +704,7 @@
 Correct Behavior: The appearance of the report should be changed to 'use percent values'</t>
         </is>
       </c>
-      <c r="H4" s="1" t="inlineStr">
+      <c r="H6" s="1" t="inlineStr">
         <is>
           <t>Buggy Behavior: the app crashes and shows a crash dialog/message: “Unfortunately, Family Finance has stopped.”
 Triggering GUI Interactions: opens the “Display” dialog and taps the “Use percent values” checkbox
@@ -630,22 +712,22 @@
 Correct Behavior: The view should switch from “view values” to “use percent values” without crashing.</t>
         </is>
       </c>
-      <c r="I4" s="1" t="inlineStr">
-        <is>
-          <t>Correct</t>
-        </is>
-      </c>
-      <c r="J4" s="1" t="inlineStr">
-        <is>
-          <t>Correct</t>
-        </is>
-      </c>
-      <c r="K4" s="1" t="inlineStr">
+      <c r="I6" s="1" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+      <c r="J6" s="1" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+      <c r="K6" s="1" t="inlineStr">
         <is>
           <t>Incomplete</t>
         </is>
       </c>
-      <c r="L4" s="1" t="inlineStr">
+      <c r="L6" s="1" t="inlineStr">
         <is>
           <t>Correct</t>
         </is>

</xml_diff>